<commit_message>
prototype for multi-lobe proposal
</commit_message>
<xml_diff>
--- a/Backend/asset-transfer-basic/application-javascript/blockchain/blockchain_hist_out.xlsx
+++ b/Backend/asset-transfer-basic/application-javascript/blockchain/blockchain_hist_out.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D42"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -956,32 +956,18 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>Sun Jan 29 2023 10:10:54 GMT+0000 (Coordinated Universal Time)</v>
+        <v>Wed Feb 01 2023 15:19:14 GMT+0000 (Coordinated Universal Time)</v>
       </c>
       <c r="C42" t="str">
         <v>commemt: Add a new use case in the ontology Manufacture, the use case called Danobat, file hash: https://github.com/tibonto/dr/archive/50d0834deba2ce791772be7932055cf1a7bb9545.zip</v>
       </c>
       <c r="D42" t="str">
-        <v>24b52a6e99fb137f72a4d92773c593ec84740ad7f8cf1ae4adcf6ea6f643e4a5</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="str">
-        <v>Sun Jan 29 2023 10:12:32 GMT+0000 (Coordinated Universal Time)</v>
-      </c>
-      <c r="C43" t="str">
-        <v>vetoProposal.OriginalID:proposal2</v>
-      </c>
-      <c r="D43" t="str">
-        <v>3353d726a1ef34867771bd67506c0115179c33ee6ce7e883a794f767dc0c7e31</v>
+        <v>3ea0b640f60ef49a3e8b7f76bb84a1523932225379b84a9f115cf4d2bb44cdb2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D42"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>